<commit_message>
incorporated working incorporation of images into reports, and also background of cards
</commit_message>
<xml_diff>
--- a/amplify/functions/process-policy-report/_report_configuration.xlsx
+++ b/amplify/functions/process-policy-report/_report_configuration.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rmiteduau-my.sharepoint.com/personal/carl_higgs_rmit_edu_au/Documents/projects/global-indicators/process/configuration/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rmiteduau-my.sharepoint.com/personal/carl_higgs_rmit_edu_au/Documents/projects/global-indicators/process/configuration/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="363" documentId="13_ncr:1_{974DC119-FBC5-4146-98A2-4FA425A99853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F80D3D92-49EA-4625-9A3C-0DA31462B0D4}"/>
+  <xr:revisionPtr revIDLastSave="368" documentId="13_ncr:1_{974DC119-FBC5-4146-98A2-4FA425A99853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B858FA20-6F52-457E-A945-5BA9DEBB829C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="policy_spatial" sheetId="1" r:id="rId1"/>
@@ -16593,7 +16593,14 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="5">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -16608,20 +16615,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -19237,8 +19230,8 @@
         <v>14</v>
       </c>
       <c r="E39">
-        <f>G38+20</f>
-        <v>126</v>
+        <f>G38+26</f>
+        <v>132</v>
       </c>
       <c r="F39">
         <f t="shared" si="7"/>
@@ -19246,7 +19239,7 @@
       </c>
       <c r="G39">
         <f t="shared" si="8"/>
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="H39" t="s">
         <v>102</v>
@@ -19298,7 +19291,7 @@
       </c>
       <c r="E40">
         <f>G39+4</f>
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="F40">
         <f t="shared" si="7"/>
@@ -19306,7 +19299,7 @@
       </c>
       <c r="G40">
         <f t="shared" si="8"/>
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="H40" t="s">
         <v>102</v>
@@ -19358,7 +19351,7 @@
       </c>
       <c r="E41">
         <f>G40+12</f>
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="F41">
         <f t="shared" si="7"/>
@@ -19366,7 +19359,7 @@
       </c>
       <c r="G41">
         <f t="shared" si="8"/>
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H41" t="s">
         <v>102</v>
@@ -19418,7 +19411,7 @@
       </c>
       <c r="E42">
         <f>G41+4</f>
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="F42">
         <f t="shared" si="7"/>
@@ -19426,7 +19419,7 @@
       </c>
       <c r="G42">
         <f t="shared" si="8"/>
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="H42" t="s">
         <v>102</v>
@@ -19478,7 +19471,7 @@
       </c>
       <c r="E43">
         <f>G42+28</f>
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="F43">
         <f t="shared" si="7"/>
@@ -19486,7 +19479,7 @@
       </c>
       <c r="G43">
         <f t="shared" si="8"/>
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="H43" t="s">
         <v>102</v>
@@ -19538,7 +19531,7 @@
       </c>
       <c r="E44">
         <f>G43+4</f>
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="F44">
         <f t="shared" si="7"/>
@@ -19546,7 +19539,7 @@
       </c>
       <c r="G44">
         <f t="shared" si="8"/>
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="H44" t="s">
         <v>102</v>
@@ -38988,15 +38981,15 @@
         <v>14</v>
       </c>
       <c r="E40">
-        <f>G39+20</f>
-        <v>114</v>
+        <f>G39+26</f>
+        <v>120</v>
       </c>
       <c r="F40">
         <v>196</v>
       </c>
       <c r="G40">
         <f t="shared" si="6"/>
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H40" t="s">
         <v>102</v>
@@ -39047,14 +39040,14 @@
       </c>
       <c r="E41">
         <f>G40+4</f>
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F41">
         <v>196</v>
       </c>
       <c r="G41">
         <f t="shared" si="6"/>
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="H41" t="s">
         <v>102</v>
@@ -39105,14 +39098,14 @@
       </c>
       <c r="E42">
         <f>G41+26</f>
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="F42">
         <v>196</v>
       </c>
       <c r="G42">
         <f t="shared" si="6"/>
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="H42" t="s">
         <v>102</v>
@@ -39163,14 +39156,14 @@
       </c>
       <c r="E43">
         <f>G42+4</f>
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="F43">
         <v>196</v>
       </c>
       <c r="G43">
         <f t="shared" si="6"/>
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="H43" t="s">
         <v>102</v>
@@ -39221,14 +39214,14 @@
       </c>
       <c r="E44">
         <f>G43+16</f>
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="F44">
         <v>196</v>
       </c>
       <c r="G44">
         <f t="shared" si="6"/>
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="H44" t="s">
         <v>102</v>
@@ -39279,14 +39272,14 @@
       </c>
       <c r="E45">
         <f>G44+4</f>
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="F45">
         <v>196</v>
       </c>
       <c r="G45">
         <f t="shared" si="6"/>
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="H45" t="s">
         <v>102</v>
@@ -46092,15 +46085,15 @@
         <v>14</v>
       </c>
       <c r="E39">
-        <f>G38+20</f>
-        <v>115</v>
+        <f>G38+26</f>
+        <v>121</v>
       </c>
       <c r="F39">
         <v>196</v>
       </c>
       <c r="G39">
         <f t="shared" si="6"/>
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="H39" t="s">
         <v>102</v>
@@ -46151,14 +46144,14 @@
       </c>
       <c r="E40">
         <f>G39+4</f>
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F40">
         <v>196</v>
       </c>
       <c r="G40">
         <f t="shared" si="6"/>
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="H40" t="s">
         <v>102</v>
@@ -46209,14 +46202,14 @@
       </c>
       <c r="E41">
         <f>G40+12</f>
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="F41">
         <v>196</v>
       </c>
       <c r="G41">
         <f t="shared" si="6"/>
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H41" t="s">
         <v>102</v>
@@ -46267,14 +46260,14 @@
       </c>
       <c r="E42">
         <f>G41+4</f>
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="F42">
         <v>196</v>
       </c>
       <c r="G42">
         <f t="shared" si="6"/>
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="H42" t="s">
         <v>102</v>
@@ -46325,14 +46318,14 @@
       </c>
       <c r="E43">
         <f>G42+28</f>
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="F43">
         <v>196</v>
       </c>
       <c r="G43">
         <f t="shared" si="6"/>
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="H43" t="s">
         <v>102</v>
@@ -46383,14 +46376,14 @@
       </c>
       <c r="E44">
         <f>G43+4</f>
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="F44">
         <v>196</v>
       </c>
       <c r="G44">
         <f t="shared" si="6"/>
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="H44" t="s">
         <v>102</v>
@@ -77391,19 +77384,14 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1:B150 B162:B1048576">
-    <cfRule type="duplicateValues" dxfId="4" priority="111"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C1:BB150 C162:BB179">
-    <cfRule type="containsBlanks" dxfId="3" priority="73">
-      <formula>LEN(TRIM(C1))=0</formula>
-    </cfRule>
+    <cfRule type="duplicateValues" dxfId="3" priority="111"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="B151:B161">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C151:BB161">
-    <cfRule type="containsBlanks" dxfId="0" priority="1">
-      <formula>LEN(TRIM(C151))=0</formula>
+  <conditionalFormatting sqref="C1:BB179">
+    <cfRule type="containsBlanks" dxfId="1" priority="1">
+      <formula>LEN(TRIM(C1))=0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -78340,7 +78328,7 @@
     <mergeCell ref="A2:A3"/>
   </mergeCells>
   <conditionalFormatting sqref="A5:A20">
-    <cfRule type="containsBlanks" dxfId="2" priority="1">
+    <cfRule type="containsBlanks" dxfId="0" priority="1">
       <formula>LEN(TRIM(A5))=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
updated settings display and image upload niceties, also tweaked report format custom box locations and custom text box setting name
</commit_message>
<xml_diff>
--- a/amplify/functions/process-policy-report/_report_configuration.xlsx
+++ b/amplify/functions/process-policy-report/_report_configuration.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://rmiteduau-my.sharepoint.com/personal/carl_higgs_rmit_edu_au/Documents/projects/global-indicators/process/configuration/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\ghsci-policy\amplify\functions\process-policy-report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="368" documentId="13_ncr:1_{974DC119-FBC5-4146-98A2-4FA425A99853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B858FA20-6F52-457E-A945-5BA9DEBB829C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5980F583-BA03-41C4-B6AC-84F54D5642C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7290" yWindow="1185" windowWidth="21600" windowHeight="11295" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="policy_spatial" sheetId="1" r:id="rId1"/>
@@ -46085,15 +46085,15 @@
         <v>14</v>
       </c>
       <c r="E39">
-        <f>G38+26</f>
-        <v>121</v>
+        <f>G38+30</f>
+        <v>125</v>
       </c>
       <c r="F39">
         <v>196</v>
       </c>
       <c r="G39">
         <f t="shared" si="6"/>
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="H39" t="s">
         <v>102</v>
@@ -46144,14 +46144,14 @@
       </c>
       <c r="E40">
         <f>G39+4</f>
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="F40">
         <v>196</v>
       </c>
       <c r="G40">
         <f t="shared" si="6"/>
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="H40" t="s">
         <v>102</v>
@@ -46201,7 +46201,7 @@
         <v>14</v>
       </c>
       <c r="E41">
-        <f>G40+12</f>
+        <f>G40+8</f>
         <v>147</v>
       </c>
       <c r="F41">
@@ -46317,15 +46317,15 @@
         <v>14</v>
       </c>
       <c r="E43">
-        <f>G42+28</f>
-        <v>189</v>
+        <f>G42+30</f>
+        <v>191</v>
       </c>
       <c r="F43">
         <v>196</v>
       </c>
       <c r="G43">
         <f t="shared" si="6"/>
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H43" t="s">
         <v>102</v>
@@ -46376,14 +46376,14 @@
       </c>
       <c r="E44">
         <f>G43+4</f>
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F44">
         <v>196</v>
       </c>
       <c r="G44">
         <f t="shared" si="6"/>
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H44" t="s">
         <v>102</v>

</xml_diff>